<commit_message>
login riuscito di alcuni link, da finire per accesso su tasti dinamici
</commit_message>
<xml_diff>
--- a/user e password per Operations.xlsx
+++ b/user e password per Operations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ytoure\Desktop\app bandi gara\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23712652-7667-4FED-B19C-156C987E62DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9177B476-8B5C-489A-B794-0F84F148C877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2295" yWindow="2295" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="61">
   <si>
     <t>REFERENTE</t>
   </si>
@@ -203,90 +203,6 @@
   </si>
   <si>
     <t>E-mail assistenza: helpdesk@pro-q.it Tel. +39 06 87 16 5516</t>
-  </si>
-  <si>
-    <t>Nokia</t>
-  </si>
-  <si>
-    <t>https://service.ariba.com/Sourcing.aw/109521010/aw?awh=r&amp;awssk=xNf5p0Ij&amp;dard=1&amp;ancdc=1#b0</t>
-  </si>
-  <si>
-    <t>claudiogare@hqe.it</t>
-  </si>
-  <si>
-    <t>TVlgal12T45!</t>
-  </si>
-  <si>
-    <t>claudio.verga@hqcon.it</t>
-  </si>
-  <si>
-    <t>Password3!</t>
-  </si>
-  <si>
-    <t>Password2!</t>
-  </si>
-  <si>
-    <t>Open Fiber</t>
-  </si>
-  <si>
-    <t>https://procurement.openfiber.it/web/login.html</t>
-  </si>
-  <si>
-    <t>hqe</t>
-  </si>
-  <si>
-    <t>Password25!</t>
-  </si>
-  <si>
-    <t>Open-Es</t>
-  </si>
-  <si>
-    <t>https://www.openes.io/it</t>
-  </si>
-  <si>
-    <t>HQengita25?</t>
-  </si>
-  <si>
-    <t>CONSORZIO HQ</t>
-  </si>
-  <si>
-    <t>Opnet</t>
-  </si>
-  <si>
-    <t>https://opnet.4buyer.it/portal</t>
-  </si>
-  <si>
-    <t>F0092A</t>
-  </si>
-  <si>
-    <t>HQengita25$</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opnet </t>
-  </si>
-  <si>
-    <t>F7453A</t>
-  </si>
-  <si>
-    <t>Milano123!</t>
-  </si>
-  <si>
-    <t>Opnet (Ex Linkem)</t>
-  </si>
-  <si>
-    <t>https://opnet.4buyer.it/Portal/</t>
-  </si>
-  <si>
-    <t>P@ssw0rd</t>
-  </si>
-  <si>
-    <t>Portale CEIT</t>
-  </si>
-  <si>
-    <t>https://ceit.vittoriarms.eu/</t>
-  </si>
-  <si>
-    <t>QTECHSRL.Utente94410</t>
   </si>
 </sst>
 </file>
@@ -851,14 +767,14 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1131,11 +1047,11 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="56" t="s">
+      <c r="I4" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="J4" s="57"/>
-      <c r="K4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="59"/>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="2"/>
@@ -1522,159 +1438,77 @@
     </row>
     <row r="18" spans="1:26" ht="15.75" customHeight="1">
       <c r="A18" s="14"/>
-      <c r="B18" s="6">
-        <v>56</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="G18" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="H18" s="16" t="s">
-        <v>40</v>
-      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="16"/>
       <c r="I18" s="15"/>
       <c r="J18" s="11"/>
       <c r="K18" s="11"/>
     </row>
     <row r="19" spans="1:26" ht="15.75" customHeight="1">
       <c r="A19" s="14"/>
-      <c r="B19" s="6">
-        <v>57</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="F19" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="H19" s="16" t="s">
-        <v>40</v>
-      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="16"/>
       <c r="I19" s="15"/>
       <c r="J19" s="11"/>
       <c r="K19" s="11"/>
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1">
       <c r="A20" s="2"/>
-      <c r="B20" s="6">
-        <v>58</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>55</v>
-      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="16"/>
       <c r="I20" s="15"/>
       <c r="J20" s="11"/>
       <c r="K20" s="11"/>
     </row>
     <row r="21" spans="1:26" ht="15.75" customHeight="1">
       <c r="A21" s="2"/>
-      <c r="B21" s="6">
-        <v>59</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="F21" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="G21" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>40</v>
-      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="16"/>
       <c r="I21" s="15"/>
       <c r="J21" s="11"/>
       <c r="K21" s="11"/>
     </row>
     <row r="22" spans="1:26" ht="15.75" customHeight="1">
       <c r="A22" s="2"/>
-      <c r="B22" s="6">
-        <v>60</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>75</v>
-      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="16"/>
       <c r="I22" s="15"/>
       <c r="J22" s="11"/>
       <c r="K22" s="11"/>
     </row>
     <row r="23" spans="1:26" ht="15.75" customHeight="1">
       <c r="A23" s="2"/>
-      <c r="B23" s="6">
-        <v>61</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>79</v>
-      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="6"/>
       <c r="H23" s="16"/>
       <c r="I23" s="11"/>
       <c r="J23" s="11"/>
@@ -1682,24 +1516,12 @@
     </row>
     <row r="24" spans="1:26" ht="15.75" customHeight="1">
       <c r="A24" s="2"/>
-      <c r="B24" s="6">
-        <v>62</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>82</v>
-      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="6"/>
       <c r="H24" s="16"/>
       <c r="I24" s="11"/>
       <c r="J24" s="11"/>
@@ -1707,22 +1529,12 @@
     </row>
     <row r="25" spans="1:26" ht="15.75" customHeight="1">
       <c r="A25" s="2"/>
-      <c r="B25" s="6">
-        <v>63</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>83</v>
-      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="11"/>
-      <c r="E25" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G25" s="36" t="s">
-        <v>85</v>
-      </c>
+      <c r="E25" s="15"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="36"/>
       <c r="H25" s="16"/>
       <c r="I25" s="11"/>
       <c r="J25" s="11"/>
@@ -1730,22 +1542,12 @@
     </row>
     <row r="26" spans="1:26" ht="15.75" customHeight="1">
       <c r="A26" s="14"/>
-      <c r="B26" s="6">
-        <v>64</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>86</v>
-      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="11"/>
       <c r="D26" s="11"/>
-      <c r="E26" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="G26" s="11" t="s">
-        <v>88</v>
-      </c>
+      <c r="E26" s="15"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
       <c r="H26" s="16"/>
       <c r="I26" s="11"/>
       <c r="J26" s="11"/>
@@ -1834,7 +1636,7 @@
       <c r="A31" s="2"/>
       <c r="B31" s="27"/>
       <c r="C31" s="28"/>
-      <c r="D31" s="59"/>
+      <c r="D31" s="56"/>
       <c r="E31" s="29"/>
       <c r="F31" s="28"/>
       <c r="G31" s="27"/>
@@ -10781,21 +10583,8 @@
     <hyperlink ref="E16" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
     <hyperlink ref="F16" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
     <hyperlink ref="E17" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="E18" r:id="rId21" location="b0" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="F18" r:id="rId22" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="E19" r:id="rId23" location="b0" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="F19" r:id="rId24" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="F20" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="E21" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="E22" r:id="rId27" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="F22" r:id="rId28" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="E23" r:id="rId29" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="E24" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="E25" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="G25" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="E26" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" r:id="rId34"/>
+  <pageSetup orientation="landscape" r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>